<commit_message>
feat: Update JSON output to include a `last_updated` timestamp and wrap data in a `data` key.
</commit_message>
<xml_diff>
--- a/alquileres.xlsx
+++ b/alquileres.xlsx
@@ -1053,7 +1053,7 @@
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="5" t="inlineStr">
         <is>
-          <t>https://casa.mercadolibre.com.uy/MLU-671466621-casa-en-barros-blancos-km-26500-de-ruta-8-a-una-cuadra-de-la-ruta-exelente-estado-_JM#polycard_client=search-desktop&amp;search_layout=grid&amp;position=1&amp;type=item&amp;float_highlight=recent_publication&amp;tracking_id=8fa80751-3c15-4442-89a9-8548f7a11feb</t>
+          <t>https://casa.mercadolibre.com.uy/MLU-671466621-casa-en-barros-blancos-km-26500-de-ruta-8-a-una-cuadra-de-la-ruta-exelente-estado-_JM#polycard_client=search-desktop&amp;search_layout=grid&amp;position=1&amp;type=item&amp;float_highlight=recent_publication&amp;tracking_id=6707838f-7741-41a1-8ed7-e7536d4cf9dc</t>
         </is>
       </c>
     </row>
@@ -1649,7 +1649,7 @@
       <c r="J16" s="2" t="inlineStr"/>
       <c r="K16" s="5" t="inlineStr">
         <is>
-          <t>https://casa.mercadolibre.com.uy/MLU-671466621-casa-en-barros-blancos-km-26500-de-ruta-8-a-una-cuadra-de-la-ruta-exelente-estado-_JM#polycard_client=search-desktop&amp;search_layout=grid&amp;position=3&amp;type=item&amp;float_highlight=recent_publication&amp;tracking_id=38afd6a9-f1c6-4d17-a892-fbbea1d29c16</t>
+          <t>https://casa.mercadolibre.com.uy/MLU-671466621-casa-en-barros-blancos-km-26500-de-ruta-8-a-una-cuadra-de-la-ruta-exelente-estado-_JM#polycard_client=search-desktop&amp;search_layout=grid&amp;position=3&amp;type=item&amp;float_highlight=recent_publication&amp;tracking_id=9ed9eb41-7aaf-4f9e-b17e-c48329c23f88</t>
         </is>
       </c>
     </row>
@@ -1686,7 +1686,7 @@
       <c r="J17" s="2" t="inlineStr"/>
       <c r="K17" s="5" t="inlineStr">
         <is>
-          <t>https://casa.mercadolibre.com.uy/MLU-1102142650-alquiler-casa-2-dormitorios-ruta-101-barros-blanco-_JM#polycard_client=search-desktop&amp;search_layout=grid&amp;position=2&amp;type=item&amp;tracking_id=38afd6a9-f1c6-4d17-a892-fbbea1d29c16</t>
+          <t>https://casa.mercadolibre.com.uy/MLU-1102142650-alquiler-casa-2-dormitorios-ruta-101-barros-blanco-_JM#polycard_client=search-desktop&amp;search_layout=grid&amp;position=2&amp;type=item&amp;tracking_id=9ed9eb41-7aaf-4f9e-b17e-c48329c23f88</t>
         </is>
       </c>
     </row>
@@ -1723,7 +1723,7 @@
       <c r="J18" s="2" t="inlineStr"/>
       <c r="K18" s="5" t="inlineStr">
         <is>
-          <t>https://casa.mercadolibre.com.uy/MLU-1203405184-alquiler-casa-2-dormitorios-barros-blancos-_JM#polycard_client=search-desktop&amp;search_layout=grid&amp;position=1&amp;type=item&amp;float_highlight=recent_publication&amp;tracking_id=38afd6a9-f1c6-4d17-a892-fbbea1d29c16</t>
+          <t>https://casa.mercadolibre.com.uy/MLU-1203405184-alquiler-casa-2-dormitorios-barros-blancos-_JM#polycard_client=search-desktop&amp;search_layout=grid&amp;position=1&amp;type=item&amp;float_highlight=recent_publication&amp;tracking_id=9ed9eb41-7aaf-4f9e-b17e-c48329c23f88</t>
         </is>
       </c>
     </row>
@@ -1760,7 +1760,7 @@
       <c r="J19" s="2" t="inlineStr"/>
       <c r="K19" s="5" t="inlineStr">
         <is>
-          <t>https://casa.mercadolibre.com.uy/MLU-1219998218-alquiler-casa-2-dormitorios-barros-blancos-_JM#polycard_client=search-desktop&amp;search_layout=grid&amp;position=4&amp;type=item&amp;float_highlight=recent_publication&amp;tracking_id=38afd6a9-f1c6-4d17-a892-fbbea1d29c16</t>
+          <t>https://casa.mercadolibre.com.uy/MLU-1219998218-alquiler-casa-2-dormitorios-barros-blancos-_JM#polycard_client=search-desktop&amp;search_layout=grid&amp;position=4&amp;type=item&amp;float_highlight=recent_publication&amp;tracking_id=9ed9eb41-7aaf-4f9e-b17e-c48329c23f88</t>
         </is>
       </c>
     </row>
@@ -1797,7 +1797,7 @@
       <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="5" t="inlineStr">
         <is>
-          <t>https://casa.mercadolibre.com.uy/MLU-1220691776-alquiler-casa-dos-dormitorios-barros-blancos-_JM#polycard_client=search-desktop&amp;search_layout=grid&amp;position=5&amp;type=item&amp;float_highlight=recent_publication&amp;tracking_id=38afd6a9-f1c6-4d17-a892-fbbea1d29c16</t>
+          <t>https://casa.mercadolibre.com.uy/MLU-1220691776-alquiler-casa-dos-dormitorios-barros-blancos-_JM#polycard_client=search-desktop&amp;search_layout=grid&amp;position=5&amp;type=item&amp;float_highlight=recent_publication&amp;tracking_id=9ed9eb41-7aaf-4f9e-b17e-c48329c23f88</t>
         </is>
       </c>
     </row>

</xml_diff>